<commit_message>
agregar total de cantidad preasignada
</commit_message>
<xml_diff>
--- a/public/375 pendientes.xlsx
+++ b/public/375 pendientes.xlsx
@@ -15,14 +15,14 @@
     <sheet name="375" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'375'!$B$8:$D$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'375'!$B$8:$E$37</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>CODIGO</t>
   </si>
@@ -40,6 +40,9 @@
   </si>
   <si>
     <t xml:space="preserve">Nº CLIENTE: </t>
+  </si>
+  <si>
+    <t>PREASIGNADO</t>
   </si>
 </sst>
 </file>
@@ -102,7 +105,10 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="6">
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -187,6 +193,10 @@
       <rgbColor rgb="00333399"/>
       <rgbColor rgb="00424242"/>
     </indexedColors>
+    <mruColors>
+      <color rgb="FF5F5F5F"/>
+      <color rgb="FF666699"/>
+    </mruColors>
   </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -210,7 +220,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>2316480</xdr:colOff>
+      <xdr:colOff>2554605</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>157503</xdr:rowOff>
     </xdr:to>
@@ -253,13 +263,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>3</xdr:col>
+      <xdr:col>4</xdr:col>
       <xdr:colOff>138925</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
+      <xdr:col>4</xdr:col>
       <xdr:colOff>1032534</xdr:colOff>
       <xdr:row>6</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
@@ -291,7 +301,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5415775" y="0"/>
+          <a:off x="6063475" y="0"/>
           <a:ext cx="893609" cy="1123950"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -305,11 +315,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A8:D37" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
-  <tableColumns count="4">
-    <tableColumn id="1" name="CODIGO" dataDxfId="2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A8:E37" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
+  <tableColumns count="5">
+    <tableColumn id="1" name="CODIGO" dataDxfId="3"/>
     <tableColumn id="2" name="DETALLE"/>
-    <tableColumn id="3" name="CANTIDAD" dataDxfId="1"/>
+    <tableColumn id="5" name="CANTIDAD" dataDxfId="2"/>
+    <tableColumn id="3" name="PREASIGNADO" dataDxfId="1"/>
     <tableColumn id="4" name="ESTADO" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium10" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -613,48 +624,49 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:F30"/>
+  <dimension ref="A2:G30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.28515625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" style="2" customWidth="1"/>
     <col min="2" max="2" width="52.7109375" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="16.28515625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="24.7109375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E2" s="1"/>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F2" s="1"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E3" s="1"/>
+      <c r="G2" s="1"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F3" s="1"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E4" s="1"/>
+      <c r="G3" s="1"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F4" s="1"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G4" s="1"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="4"/>
-      <c r="E5" s="1"/>
       <c r="F5" s="1"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G5" s="1"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B6" s="5"/>
-      <c r="E6" s="1"/>
       <c r="F6" s="1"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E7" s="1"/>
+      <c r="G6" s="1"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F7" s="1"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G7" s="1"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>0</v>
       </c>
@@ -665,98 +677,101 @@
         <v>2</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E8" s="1"/>
       <c r="F8" s="1"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E9" s="1"/>
+      <c r="G8" s="1"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F9" s="1"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E10" s="1"/>
+      <c r="G9" s="1"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F10" s="1"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E11" s="1"/>
+      <c r="G10" s="1"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F11" s="1"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E12" s="1"/>
+      <c r="G11" s="1"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F12" s="1"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E13" s="1"/>
+      <c r="G12" s="1"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F13" s="1"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E14" s="1"/>
+      <c r="G13" s="1"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F14" s="1"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E15" s="1"/>
+      <c r="G14" s="1"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F15" s="1"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E16" s="1"/>
+      <c r="G15" s="1"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F16" s="1"/>
-    </row>
-    <row r="17" spans="5:6" x14ac:dyDescent="0.2">
-      <c r="E17" s="1"/>
+      <c r="G16" s="1"/>
+    </row>
+    <row r="17" spans="6:7" x14ac:dyDescent="0.2">
       <c r="F17" s="1"/>
-    </row>
-    <row r="18" spans="5:6" x14ac:dyDescent="0.2">
-      <c r="E18" s="1"/>
+      <c r="G17" s="1"/>
+    </row>
+    <row r="18" spans="6:7" x14ac:dyDescent="0.2">
       <c r="F18" s="1"/>
-    </row>
-    <row r="19" spans="5:6" x14ac:dyDescent="0.2">
-      <c r="E19" s="1"/>
+      <c r="G18" s="1"/>
+    </row>
+    <row r="19" spans="6:7" x14ac:dyDescent="0.2">
       <c r="F19" s="1"/>
-    </row>
-    <row r="20" spans="5:6" x14ac:dyDescent="0.2">
-      <c r="E20" s="1"/>
+      <c r="G19" s="1"/>
+    </row>
+    <row r="20" spans="6:7" x14ac:dyDescent="0.2">
       <c r="F20" s="1"/>
-    </row>
-    <row r="21" spans="5:6" x14ac:dyDescent="0.2">
-      <c r="E21" s="1"/>
+      <c r="G20" s="1"/>
+    </row>
+    <row r="21" spans="6:7" x14ac:dyDescent="0.2">
       <c r="F21" s="1"/>
-    </row>
-    <row r="22" spans="5:6" x14ac:dyDescent="0.2">
-      <c r="E22" s="1"/>
+      <c r="G21" s="1"/>
+    </row>
+    <row r="22" spans="6:7" x14ac:dyDescent="0.2">
       <c r="F22" s="1"/>
-    </row>
-    <row r="23" spans="5:6" x14ac:dyDescent="0.2">
-      <c r="E23" s="1"/>
+      <c r="G22" s="1"/>
+    </row>
+    <row r="23" spans="6:7" x14ac:dyDescent="0.2">
       <c r="F23" s="1"/>
-    </row>
-    <row r="24" spans="5:6" x14ac:dyDescent="0.2">
-      <c r="E24" s="1"/>
+      <c r="G23" s="1"/>
+    </row>
+    <row r="24" spans="6:7" x14ac:dyDescent="0.2">
       <c r="F24" s="1"/>
-    </row>
-    <row r="25" spans="5:6" x14ac:dyDescent="0.2">
-      <c r="E25" s="1"/>
+      <c r="G24" s="1"/>
+    </row>
+    <row r="25" spans="6:7" x14ac:dyDescent="0.2">
       <c r="F25" s="1"/>
-    </row>
-    <row r="26" spans="5:6" x14ac:dyDescent="0.2">
-      <c r="E26" s="1"/>
+      <c r="G25" s="1"/>
+    </row>
+    <row r="26" spans="6:7" x14ac:dyDescent="0.2">
       <c r="F26" s="1"/>
-    </row>
-    <row r="27" spans="5:6" x14ac:dyDescent="0.2">
-      <c r="E27" s="1"/>
+      <c r="G26" s="1"/>
+    </row>
+    <row r="27" spans="6:7" x14ac:dyDescent="0.2">
       <c r="F27" s="1"/>
-    </row>
-    <row r="28" spans="5:6" x14ac:dyDescent="0.2">
-      <c r="E28" s="1"/>
+      <c r="G27" s="1"/>
+    </row>
+    <row r="28" spans="6:7" x14ac:dyDescent="0.2">
       <c r="F28" s="1"/>
-    </row>
-    <row r="29" spans="5:6" x14ac:dyDescent="0.2">
-      <c r="E29" s="1"/>
+      <c r="G28" s="1"/>
+    </row>
+    <row r="29" spans="6:7" x14ac:dyDescent="0.2">
       <c r="F29" s="1"/>
-    </row>
-    <row r="30" spans="5:6" x14ac:dyDescent="0.2">
-      <c r="E30" s="1"/>
+      <c r="G29" s="1"/>
+    </row>
+    <row r="30" spans="6:7" x14ac:dyDescent="0.2">
       <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
     </row>
   </sheetData>
   <sortState ref="A9:D37">

</xml_diff>